<commit_message>
Stage 3: input fuse F1 becomes a not-fitted option, R96 link (refs #3)
0456025.ER is rated 72 VDC, below the 79.2 V maximum input, and no
>=25 A SMD fuse rated >=100 VDC was found. Per review decision the
LM5069 circuit breaker is the eFuse; F1 keeps its NANO2 456 footprint
(DNP) and R96 (Bourns CSS2H-2512C-000, <0.1 mOhm, 100 A) links it.
Adds the R_2512_CSS2H footprint; BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/PCB_BOM.xlsx
+++ b/bom/PCB_BOM.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Original (report BOM)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$96</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>D_SOD-323</t>
+          <t>SOT-323_SC-70</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -1796,22 +1796,22 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>FB1</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>25A</t>
+          <t>600R@100MHz</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0456025.ER</t>
+          <t>BLM18KG601SN1D</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Littelfuse</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1821,20 +1821,16 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>C315877</t>
+          <t>C85833</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Fuse_Littelfuse_NANO2_456</t>
+          <t>L_0603_1608Metric</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>Custom footprint, drawn in Stage 3</t>
-        </is>
-      </c>
+      <c r="M29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1845,22 +1841,22 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>FB1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>600R@100MHz</t>
+          <t>DC+ 72V</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BLM18KG601SN1D</t>
+          <t>74650194R</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1868,14 +1864,10 @@
         <f>IF(H30="","",H30*B30)</f>
         <v/>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>C85833</t>
-        </is>
-      </c>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>L_0603_1608Metric</t>
+          <t>Wurth_REDCUBE_74650194</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
@@ -1890,12 +1882,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DC+ 72V</t>
+          <t>VOUT+</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1920,11 +1912,7 @@
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>Custom footprint, drawn in Stage 3</t>
-        </is>
-      </c>
+      <c r="M31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1935,12 +1923,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>VOUT+</t>
+          <t>DC- return</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1965,11 +1953,7 @@
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>Custom footprint, drawn in Stage 3</t>
-        </is>
-      </c>
+      <c r="M32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1980,39 +1964,50 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DC- return</t>
+          <t>RACK I/O Nano-Fit</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>74650194R</t>
+          <t>105313-1206</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>Molex</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>WM14975-ND</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>2.54</v>
+      </c>
       <c r="I33">
         <f>IF(H33="","",H33*B33)</f>
         <v/>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>C17656275</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Wurth_REDCUBE_74650194</t>
+          <t>Molex_Nano-Fit_105313-xx06_1x06_P2.50mm_Horizontal</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Custom footprint, drawn in Stage 3</t>
+          <t>Required part (CLAUDE.md section 4)</t>
         </is>
       </c>
     </row>
@@ -2025,17 +2020,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RACK I/O Nano-Fit</t>
+          <t>FAN Micro-Fit</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>105313-1206</t>
+          <t>43650-0400</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2043,34 +2038,23 @@
           <t>Molex</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>WM14975-ND</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
-        <v>2.54</v>
-      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="I34">
         <f>IF(H34="","",H34*B34)</f>
         <v/>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>C17656275</t>
+          <t>C277684</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Molex_Nano-Fit_105313-xx06_1x06_P2.50mm_Horizontal</t>
+          <t>Molex_Micro-Fit_3.0_43650-0400_1x04_P3.00mm_Horizontal</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>Required part (CLAUDE.md section 4)</t>
-        </is>
-      </c>
+      <c r="M34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2081,22 +2065,22 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FAN Micro-Fit</t>
+          <t>VOUT-</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>43650-0400</t>
+          <t>74650194R</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -2104,14 +2088,10 @@
         <f>IF(H35="","",H35*B35)</f>
         <v/>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>C277684</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Molex_Micro-Fit_3.0_43650-0400_1x04_P3.00mm_Horizontal</t>
+          <t>Wurth_REDCUBE_74650194</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
@@ -2126,25 +2106,32 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>VOUT-</t>
+          <t>ERUC23-3R2K</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>74650194R</t>
+          <t>ERUC23-3R2K</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>TDK</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>495-ERUC23-3R2KCT-ND</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>8.960000000000001</v>
+      </c>
       <c r="I36">
         <f>IF(H36="","",H36*B36)</f>
         <v/>
@@ -2152,13 +2139,13 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Wurth_REDCUBE_74650194</t>
+          <t>TDK_ERUC23</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Custom footprint, drawn in Stage 3</t>
+          <t>Required part (CLAUDE.md section 4); Custom footprint, drawn in Stage 3</t>
         </is>
       </c>
     </row>
@@ -2171,32 +2158,25 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ERUC23-3R2K</t>
+          <t>33uH</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ERUC23-3R2K</t>
+          <t>XAL7070-333MEB</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>TDK</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>495-ERUC23-3R2KCT-ND</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>8.960000000000001</v>
-      </c>
+          <t>Coilcraft</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="I37">
         <f>IF(H37="","",H37*B37)</f>
         <v/>
@@ -2204,15 +2184,11 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>TDK_ERUC23</t>
+          <t>L_Coilcraft_XAL7070-XXX</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>Required part (CLAUDE.md section 4); Custom footprint, drawn in Stage 3</t>
-        </is>
-      </c>
+      <c r="M37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2223,220 +2199,224 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>33uH</t>
+          <t>NME1S0505SC</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>XAL7070-333MEB</t>
+          <t>NME1S0505SC</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Coilcraft</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>Murata</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>811-NME1S0505SC-ND</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>1.86</v>
+      </c>
       <c r="I38">
         <f>IF(H38="","",H38*B38)</f>
         <v/>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>C39128444</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>L_Coilcraft_XAL7070-XXX</t>
+          <t>Murata_NME1S_SIP-4</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Required part (CLAUDE.md section 4)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>Q1, Q2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>NME1S0505SC</t>
+          <t>IPT015N10N5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NME1S0505SC</t>
+          <t>IPT015N10N5</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Murata</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>811-NME1S0505SC-ND</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>1.86</v>
-      </c>
+          <t>Infineon</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="I39">
         <f>IF(H39="","",H39*B39)</f>
         <v/>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>C39128444</t>
+          <t>C108964</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Murata_NME1S_SIP-4</t>
+          <t>Infineon_PG-HSOF-8-1</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>Required part (CLAUDE.md section 4); Custom footprint, drawn in Stage 3</t>
-        </is>
-      </c>
+      <c r="M39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Q1, Q2</t>
+          <t>Q3, Q4, Q5, Q6</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>IPT015N10N5</t>
+          <t>EPC2304</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>IPT015N10N5</t>
+          <t>EPC2304</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>EPC</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>917-EPC2304CT-ND</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>9.050000000000001</v>
+      </c>
       <c r="I40">
         <f>IF(H40="","",H40*B40)</f>
         <v/>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>C108964</t>
+          <t>C6549215</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Infineon_PG-HSOF-8-1</t>
+          <t>EPC2304_QFN-7_3x5mm</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Required part (CLAUDE.md section 4); Custom footprint, drawn in Stage 3</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Q3, Q4, Q5, Q6</t>
+          <t>Q7, Q8</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EPC2304</t>
+          <t>2N7002</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>EPC2304</t>
+          <t>2N7002LT1G</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>EPC</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>917-EPC2304CT-ND</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>9.050000000000001</v>
-      </c>
+          <t>onsemi</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="I41">
         <f>IF(H41="","",H41*B41)</f>
         <v/>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>C6549215</t>
+          <t>C16338</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>EPC2304_QFN-7_3x5mm</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>Required part (CLAUDE.md section 4); Custom footprint, drawn in Stage 3</t>
-        </is>
-      </c>
+      <c r="M41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Q7, Q8</t>
+          <t>R1, R2, R3, R4</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2N7002</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2N7002LT1G</t>
+          <t>RC0603FR-0751KL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -2444,14 +2424,10 @@
         <f>IF(H42="","",H42*B42)</f>
         <v/>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>C16338</t>
-        </is>
-      </c>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
@@ -2462,21 +2438,21 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>R1, R2, R3, R4</t>
+          <t>R9, R10</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>RC0603FR-0751KL</t>
+          <t>RC0603FR-074R7L</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2507,17 +2483,17 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>R9, R10</t>
+          <t>R13, R14</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>RC0603FR-074R7L</t>
+          <t>RC0603FR-075R6L</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2548,17 +2524,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>R13, R14</t>
+          <t>R15, R16</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>RC0603FR-075R6L</t>
+          <t>RC0603FR-072RL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2589,17 +2565,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>R15, R16</t>
+          <t>R21, R22</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6.04k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>RC0603FR-072RL</t>
+          <t>RC0603FR-076K04L</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2630,17 +2606,17 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>R21, R22</t>
+          <t>R27, R28</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>6.04k</t>
+          <t>22.6k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>RC0603FR-076K04L</t>
+          <t>RC0603FR-0722K6L</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2667,21 +2643,21 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>R27, R28</t>
+          <t>R29, R30, R48, R52, R53, R55, R58, R61, R62, R81, R84, R91, R93, R94, R95</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>22.6k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>RC0603FR-0722K6L</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2708,21 +2684,21 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>R29, R30, R48, R52, R53, R55, R58, R61, R62, R81, R84, R91, R93, R94, R95</t>
+          <t>R31, R32, R33, R34, R44</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603FR-0710RL</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2749,21 +2725,21 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>R31, R32, R33, R34, R44</t>
+          <t>R40</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5.49k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>RC0603FR-0710RL</t>
+          <t>RC0603FR-075K49L</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2794,17 +2770,17 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>R40</t>
+          <t>R41</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5.49k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>RC0603FR-075K49L</t>
+          <t>RC0603FR-071ML</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2835,17 +2811,17 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>R41</t>
+          <t>R43</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>330</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>RC0603FR-071ML</t>
+          <t>RC0603FR-07330RL</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2876,17 +2852,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>R43</t>
+          <t>R45</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>95.3k</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>RC0603FR-07330RL</t>
+          <t>RC1206FR-0795K3L</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2902,7 +2878,7 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_1206_3216Metric</t>
         </is>
       </c>
       <c r="L53" t="inlineStr"/>
@@ -2917,17 +2893,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>R45</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>95.3k</t>
+          <t>4.12k</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>RC1206FR-0795K3L</t>
+          <t>RC0603FR-074K12L</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2943,7 +2919,7 @@
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>R_1206_3216Metric</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L54" t="inlineStr"/>
@@ -2958,17 +2934,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>R46</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>4.12k</t>
+          <t>13.0k</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>RC0603FR-074K12L</t>
+          <t>RC0603FR-0713KL</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2999,22 +2975,22 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>R47</t>
+          <t>R49</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>13.0k</t>
+          <t>649k 0.1%</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>RC0603FR-0713KL</t>
+          <t>ERA-8AEB6493V</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -3025,7 +3001,7 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_1206_3216Metric</t>
         </is>
       </c>
       <c r="L56" t="inlineStr"/>
@@ -3036,21 +3012,21 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>R49</t>
+          <t>R50, R65, R69, R71</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>649k 0.1%</t>
+          <t>10.0k 0.1%</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ERA-8AEB6493V</t>
+          <t>ERA-3AEB1002V</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3066,7 +3042,7 @@
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>R_1206_3216Metric</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L57" t="inlineStr"/>
@@ -3077,26 +3053,26 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>R50, R65, R69, R71</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.0k 0.1%</t>
+          <t>1.69M</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ERA-3AEB1002V</t>
+          <t>RC0603FR-071M69L</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
@@ -3122,17 +3098,17 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>R54</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>1.69M</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>RC0603FR-071M69L</t>
+          <t>RC1206FR-07200KL</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3148,7 +3124,7 @@
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_1206_3216Metric</t>
         </is>
       </c>
       <c r="L59" t="inlineStr"/>
@@ -3163,17 +3139,17 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>R54</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>32.4k</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>RC1206FR-07200KL</t>
+          <t>RC0603FR-0732K4L</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3189,7 +3165,7 @@
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>R_1206_3216Metric</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L60" t="inlineStr"/>
@@ -3204,17 +3180,17 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R57</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>32.4k</t>
+          <t>33.2k</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>RC0603FR-0732K4L</t>
+          <t>RC0603FR-0733K2L</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3241,21 +3217,21 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>R57</t>
+          <t>R59, R86, R87</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>33.2k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>RC0603FR-0733K2L</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3282,21 +3258,21 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>R59, R86, R87</t>
+          <t>R60</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>25.5k</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-0725K5L</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3327,22 +3303,22 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>R60</t>
+          <t>R64</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>25.5k</t>
+          <t>290k 0.1%</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>RC0603FR-0725K5L</t>
+          <t>ERA-3AEB2903V</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
@@ -3368,22 +3344,22 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>R64</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>290k 0.1%</t>
+          <t>26.1k</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ERA-3AEB2903V</t>
+          <t>RC0603FR-0726K1L</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
@@ -3405,21 +3381,21 @@
         <v>65</v>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>R66</t>
+          <t>R67, R68</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>26.1k</t>
+          <t>52.3k</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>RC0603FR-0726K1L</t>
+          <t>RC0603FR-0752K3L</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3450,22 +3426,22 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>R67, R68</t>
+          <t>R70, R72</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>52.3k</t>
+          <t>5.97k 0.1%</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>RC0603FR-0752K3L</t>
+          <t>ERA-3AEB5971V</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
@@ -3487,21 +3463,21 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>R70, R72</t>
+          <t>R73, R75, R77, R79</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>5.97k 0.1%</t>
+          <t>7.50k 0.1%</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ERA-3AEB5971V</t>
+          <t>ERA-3AEB7501V</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3532,17 +3508,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>R73, R75, R77, R79</t>
+          <t>R74, R76, R78, R80</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7.50k 0.1%</t>
+          <t>2.67k 0.1%</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ERA-3AEB7501V</t>
+          <t>ERA-3AEB2671V</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3569,26 +3545,26 @@
         <v>69</v>
       </c>
       <c r="B70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>R74, R76, R78, R80</t>
+          <t>R82, R88</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2.67k 0.1%</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ERA-3AEB2671V</t>
+          <t>RC0603FR-071KL</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
@@ -3610,21 +3586,21 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>R82, R88</t>
+          <t>R83</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>RC0603FR-071KL</t>
+          <t>RC0603FR-0720KL</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3655,17 +3631,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>R83</t>
+          <t>R85</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>11.8k</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>RC0603FR-0720KL</t>
+          <t>RC0603FR-0711K8L</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3692,21 +3668,21 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>R85</t>
+          <t>R89, R90</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>11.8k</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>RC0603FR-0711K8L</t>
+          <t>RC0603FR-071K5L</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3733,21 +3709,21 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>R89, R90</t>
+          <t>R92</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>RC0603FR-071K5L</t>
+          <t>RC0603FR-07100RL</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3778,22 +3754,22 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>R92</t>
+          <t>R96</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0R 100A</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>RC0603FR-07100RL</t>
+          <t>CSS2H-2512C-000</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
@@ -3804,11 +3780,15 @@
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_2512_CSS2H</t>
         </is>
       </c>
       <c r="L75" t="inlineStr"/>
-      <c r="M75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>Custom footprint, drawn in Stage 3</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4598,28 +4578,24 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>R23, R24, R25, R26</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>FUSE OPT</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>RC1206FR-072R2L</t>
-        </is>
-      </c>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
+          <t>not fitted</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr"/>
       <c r="G93" s="3" t="inlineStr"/>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3">
@@ -4629,7 +4605,7 @@
       <c r="J93" s="3" t="inlineStr"/>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>R_1206_3216Metric</t>
+          <t>Fuse_Littelfuse_NANO2_456</t>
         </is>
       </c>
       <c r="L93" s="3" t="inlineStr">
@@ -4639,7 +4615,7 @@
       </c>
       <c r="M93" s="4" t="inlineStr">
         <is>
-          <t>DNP: footprint only</t>
+          <t>Custom footprint, drawn in Stage 3; DNP: footprint only</t>
         </is>
       </c>
     </row>
@@ -4648,21 +4624,21 @@
         <v>93</v>
       </c>
       <c r="B94" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R23, R24, R25, R26</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>RC0603JR-070RL</t>
+          <t>RC1206FR-072R2L</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -4679,7 +4655,7 @@
       <c r="J94" s="3" t="inlineStr"/>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_1206_3216Metric</t>
         </is>
       </c>
       <c r="L94" s="3" t="inlineStr">
@@ -4702,17 +4678,17 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603JR-070RL</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
@@ -4744,36 +4720,86 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="n"/>
-      <c r="B96" s="5">
-        <f>SUM(B2:B95)</f>
-        <v/>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
+      <c r="A96" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>R63</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>RC0603FR-0710KL</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr"/>
+      <c r="H96" s="3" t="n"/>
+      <c r="I96" s="3">
+        <f>IF(H96="","",H96*B96)</f>
+        <v/>
+      </c>
+      <c r="J96" s="3" t="inlineStr"/>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>R_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t>DNP: footprint only</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n"/>
+      <c r="B97" s="5">
+        <f>SUM(B2:B96)</f>
+        <v/>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>parts (incl. DNP)</t>
         </is>
       </c>
-      <c r="D96" s="5" t="n"/>
-      <c r="E96" s="5" t="n"/>
-      <c r="F96" s="5" t="n"/>
-      <c r="G96" s="5" t="n"/>
-      <c r="H96" s="5" t="inlineStr">
+      <c r="D97" s="5" t="n"/>
+      <c r="E97" s="5" t="n"/>
+      <c r="F97" s="5" t="n"/>
+      <c r="G97" s="5" t="n"/>
+      <c r="H97" s="5" t="inlineStr">
         <is>
           <t>Known total:</t>
         </is>
       </c>
-      <c r="I96" s="5">
-        <f>SUM(I2:I95)</f>
-        <v/>
-      </c>
-      <c r="J96" s="5" t="n"/>
-      <c r="K96" s="5" t="n"/>
-      <c r="L96" s="5" t="n"/>
-      <c r="M96" s="5" t="n"/>
+      <c r="I97" s="5">
+        <f>SUM(I2:I96)</f>
+        <v/>
+      </c>
+      <c r="J97" s="5" t="n"/>
+      <c r="K97" s="5" t="n"/>
+      <c r="L97" s="5" t="n"/>
+      <c r="M97" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M95"/>
+  <autoFilter ref="A1:M96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>